<commit_message>
Fix campaign UTM parity and worksheet funnel-stage labels
</commit_message>
<xml_diff>
--- a/deliverables/sentinel-campaign/cash-flow-worksheet.xlsx
+++ b/deliverables/sentinel-campaign/cash-flow-worksheet.xlsx
@@ -261,7 +261,7 @@
     <t>Illustrative 6 × $17.99 = $107.94 before taxes, refunds, fees, or expenses.</t>
   </si>
   <si>
-    <t>Optional checkout → paid-order conversion assumption</t>
+    <t>Optional checkout → paid-order conversion rate assumption</t>
   </si>
   <si>
     <t>Optional input</t>
@@ -270,16 +270,16 @@
     <t>Leave blank unless a measured, channel-specific assumption is intentionally used.</t>
   </si>
   <si>
-    <t>Illustrative visitors needed at optional conversion</t>
-  </si>
-  <si>
-    <t>Blank until the optional assumption is entered; this is not an actual result.</t>
+    <t>Illustrative checkout clicks required at optional checkout → paid-order rate</t>
+  </si>
+  <si>
+    <t>Blank until the optional rate is entered; this is checkout clicks required, not a website visitor count or actual result.</t>
   </si>
   <si>
     <t>Guardrail</t>
   </si>
   <si>
-    <t>Do not use this scenario to backfill actual orders, visitors, conversion, revenue, or cash. Actual paid orders come from sales records; purchases are not attributed from pageviews.</t>
+    <t>Do not use this scenario to backfill actual orders, checkout clicks, visitors, conversion, revenue, or cash. The optional rate yields checkout clicks required only; it does not estimate website visitors. Actual paid orders come from sales records; purchases are not attributed from pageviews.</t>
   </si>
   <si>
     <t>Weekly review — measurement and reconciliation</t>

</xml_diff>